<commit_message>
Code Committed fr POM Project
</commit_message>
<xml_diff>
--- a/src/test/resources/com/ab/excel/TestData.xlsx
+++ b/src/test/resources/com/ab/excel/TestData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
   <si>
     <t>Username</t>
   </si>
@@ -24,28 +24,19 @@
     <t>Password</t>
   </si>
   <si>
-    <t>priyank.sharma@awarebase.com</t>
-  </si>
-  <si>
-    <t>Pass@Pass@123</t>
-  </si>
-  <si>
     <t>Runmode</t>
   </si>
   <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>LoginTest</t>
-  </si>
-  <si>
-    <t>zz@test.tina5s.com</t>
-  </si>
-  <si>
-    <t>New_Record</t>
-  </si>
-  <si>
     <t>Testcase</t>
+  </si>
+  <si>
+    <t>priyank25sharma@yahoo.co.in</t>
+  </si>
+  <si>
+    <t>Test#123</t>
+  </si>
+  <si>
+    <t>Login_test</t>
   </si>
   <si>
     <t>N</t>
@@ -55,7 +46,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -74,6 +65,12 @@
     <font>
       <sz val="10"/>
       <color rgb="FF1290C3"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF17C6A3"/>
       <name val="Consolas"/>
       <family val="3"/>
     </font>
@@ -99,10 +96,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -405,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
@@ -425,61 +423,29 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
+      <c r="B3" s="3" t="s">
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>10</v>
-      </c>
+      <c r="B4" s="1"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
+      <c r="A6" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
@@ -493,10 +459,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -504,16 +470,11 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
+      <c r="A3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>